<commit_message>
Refactor event study plotting and add new outputs
Rewrote and expanded R event study plotting code in .Rhistory to generate improved event study plots with custom color schemes and confidence bands, saving new output images. Added code to generate and save event study plots for both controls and simple models, and included new data and result files for event study analysis. Removed old event study plot and reorganized output files into a new directory structure.
</commit_message>
<xml_diff>
--- a/data/controles_results/difmedias_controles_baselines_fixed_2019.xlsx
+++ b/data/controles_results/difmedias_controles_baselines_fixed_2019.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="252" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="252" uniqueCount="113">
   <si>
     <t/>
   </si>
@@ -75,10 +75,10 @@
     <t>N</t>
   </si>
   <si>
-    <t>835</t>
-  </si>
-  <si>
-    <t>747</t>
+    <t>832</t>
+  </si>
+  <si>
+    <t>744</t>
   </si>
   <si>
     <t xml:space="preserve"> (1) </t>
@@ -90,43 +90,43 @@
     <t>Mean/(SE)</t>
   </si>
   <si>
-    <t>78594.207</t>
-  </si>
-  <si>
-    <t>(2015.555)</t>
-  </si>
-  <si>
-    <t>470.168</t>
-  </si>
-  <si>
-    <t>(10.089)</t>
-  </si>
-  <si>
-    <t>73469.612</t>
-  </si>
-  <si>
-    <t>(1894.266)</t>
-  </si>
-  <si>
-    <t>485.354</t>
-  </si>
-  <si>
-    <t>(10.662)</t>
-  </si>
-  <si>
-    <t>3.503</t>
+    <t>78609.681</t>
+  </si>
+  <si>
+    <t>(2020.049)</t>
+  </si>
+  <si>
+    <t>471.380</t>
+  </si>
+  <si>
+    <t>(10.101)</t>
+  </si>
+  <si>
+    <t>73502.471</t>
+  </si>
+  <si>
+    <t>(1897.671)</t>
+  </si>
+  <si>
+    <t>486.623</t>
+  </si>
+  <si>
+    <t>(10.675)</t>
+  </si>
+  <si>
+    <t>3.505</t>
   </si>
   <si>
     <t>(0.014)</t>
   </si>
   <si>
-    <t>1.941</t>
+    <t>1.928</t>
   </si>
   <si>
     <t>(0.087)</t>
   </si>
   <si>
-    <t>89.440</t>
+    <t>89.434</t>
   </si>
   <si>
     <t>(0.138)</t>
@@ -135,10 +135,10 @@
     <t>1.05e+06</t>
   </si>
   <si>
-    <t>(21241.687)</t>
-  </si>
-  <si>
-    <t>2.818</t>
+    <t>(21264.344)</t>
+  </si>
+  <si>
+    <t>2.814</t>
   </si>
   <si>
     <t>(0.043)</t>
@@ -147,46 +147,46 @@
     <t>2.79e+11</t>
   </si>
   <si>
-    <t>(7.70e+09)</t>
-  </si>
-  <si>
-    <t>3.88e+11</t>
-  </si>
-  <si>
-    <t>(6.94e+09)</t>
-  </si>
-  <si>
-    <t>0.528</t>
+    <t>(7.71e+09)</t>
+  </si>
+  <si>
+    <t>3.87e+11</t>
+  </si>
+  <si>
+    <t>(6.96e+09)</t>
+  </si>
+  <si>
+    <t>0.526</t>
   </si>
   <si>
     <t>(0.017)</t>
   </si>
   <si>
-    <t>4.111</t>
+    <t>4.106</t>
   </si>
   <si>
     <t>(0.102)</t>
   </si>
   <si>
-    <t>0.925</t>
+    <t>0.924</t>
   </si>
   <si>
     <t>(0.009)</t>
   </si>
   <si>
-    <t>3.314</t>
+    <t>3.312</t>
   </si>
   <si>
     <t>(0.048)</t>
   </si>
   <si>
-    <t>2.792</t>
-  </si>
-  <si>
-    <t>(0.052)</t>
-  </si>
-  <si>
-    <t>61</t>
+    <t>2.789</t>
+  </si>
+  <si>
+    <t>(0.053)</t>
+  </si>
+  <si>
+    <t>64</t>
   </si>
   <si>
     <t xml:space="preserve"> (2) </t>
@@ -195,79 +195,82 @@
     <t>1</t>
   </si>
   <si>
-    <t>55442.590</t>
-  </si>
-  <si>
-    <t>(7020.198)</t>
-  </si>
-  <si>
-    <t>397.286</t>
-  </si>
-  <si>
-    <t>(41.802)</t>
-  </si>
-  <si>
-    <t>51743.492</t>
-  </si>
-  <si>
-    <t>(6719.192)</t>
-  </si>
-  <si>
-    <t>411.027</t>
-  </si>
-  <si>
-    <t>(44.380)</t>
-  </si>
-  <si>
-    <t>3.153</t>
-  </si>
-  <si>
-    <t>(0.059)</t>
-  </si>
-  <si>
-    <t>3.803</t>
-  </si>
-  <si>
-    <t>(0.352)</t>
-  </si>
-  <si>
-    <t>92.055</t>
-  </si>
-  <si>
-    <t>(0.424)</t>
+    <t>56326.656</t>
+  </si>
+  <si>
+    <t>(6848.411)</t>
+  </si>
+  <si>
+    <t>384.947</t>
+  </si>
+  <si>
+    <t>(40.452)</t>
+  </si>
+  <si>
+    <t>52334.734</t>
+  </si>
+  <si>
+    <t>(6577.739)</t>
+  </si>
+  <si>
+    <t>398.010</t>
+  </si>
+  <si>
+    <t>(42.937)</t>
+  </si>
+  <si>
+    <t>3.155</t>
+  </si>
+  <si>
+    <t>(0.058)</t>
+  </si>
+  <si>
+    <t>3.891</t>
+  </si>
+  <si>
+    <t>(0.345)</t>
+  </si>
+  <si>
+    <t>92.015</t>
+  </si>
+  <si>
+    <t>(0.419)</t>
   </si>
   <si>
     <t>1.41e+06</t>
   </si>
   <si>
-    <t>(88739.694)</t>
+    <t>(86334.338)</t>
   </si>
   <si>
     <t>3.671</t>
   </si>
   <si>
-    <t>(0.141)</t>
-  </si>
-  <si>
-    <t>3.17e+11</t>
-  </si>
-  <si>
-    <t>(3.37e+10)</t>
-  </si>
-  <si>
-    <t>3.43e+11</t>
-  </si>
-  <si>
-    <t>(2.54e+10)</t>
-  </si>
-  <si>
-    <t>0.836</t>
-  </si>
-  <si>
-    <t>6.721</t>
-  </si>
-  <si>
-    <t>(0.550)</t>
+    <t>(0.137)</t>
+  </si>
+  <si>
+    <t>3.16e+11</t>
+  </si>
+  <si>
+    <t>(3.29e+10)</t>
+  </si>
+  <si>
+    <t>3.51e+11</t>
+  </si>
+  <si>
+    <t>(2.48e+10)</t>
+  </si>
+  <si>
+    <t>0.844</t>
+  </si>
+  <si>
+    <t>(0.046)</t>
+  </si>
+  <si>
+    <t>6.672</t>
+  </si>
+  <si>
+    <t>(0.536)</t>
   </si>
   <si>
     <t>1.000</t>
@@ -276,16 +279,16 @@
     <t>(0.000)</t>
   </si>
   <si>
-    <t>3.585</t>
-  </si>
-  <si>
-    <t>(0.041)</t>
-  </si>
-  <si>
-    <t>3.660</t>
-  </si>
-  <si>
-    <t>(0.092)</t>
+    <t>3.597</t>
+  </si>
+  <si>
+    <t>(0.040)</t>
+  </si>
+  <si>
+    <t>3.656</t>
+  </si>
+  <si>
+    <t>(0.088)</t>
   </si>
   <si>
     <t>896</t>
@@ -303,49 +306,49 @@
     <t>Mean difference</t>
   </si>
   <si>
-    <t>-2.32e+04***</t>
-  </si>
-  <si>
-    <t>-72.882*</t>
-  </si>
-  <si>
-    <t>-2.17e+04***</t>
-  </si>
-  <si>
-    <t>-74.327*</t>
+    <t>-2.23e+04***</t>
+  </si>
+  <si>
+    <t>-86.433**</t>
+  </si>
+  <si>
+    <t>-2.12e+04***</t>
+  </si>
+  <si>
+    <t>-88.614**</t>
   </si>
   <si>
     <t>-0.350***</t>
   </si>
   <si>
-    <t>1.862***</t>
-  </si>
-  <si>
-    <t>2.615***</t>
-  </si>
-  <si>
-    <t>3.60e+05***</t>
-  </si>
-  <si>
-    <t>0.853***</t>
-  </si>
-  <si>
-    <t>3.79e+10</t>
-  </si>
-  <si>
-    <t>-4.48e+10*</t>
-  </si>
-  <si>
-    <t>0.308***</t>
-  </si>
-  <si>
-    <t>2.610***</t>
-  </si>
-  <si>
-    <t>0.075**</t>
-  </si>
-  <si>
-    <t>0.271</t>
+    <t>1.963***</t>
+  </si>
+  <si>
+    <t>2.581***</t>
+  </si>
+  <si>
+    <t>3.61e+05***</t>
+  </si>
+  <si>
+    <t>0.857***</t>
+  </si>
+  <si>
+    <t>3.64e+10</t>
+  </si>
+  <si>
+    <t>-3.64e+10</t>
+  </si>
+  <si>
+    <t>0.317***</t>
+  </si>
+  <si>
+    <t>2.566***</t>
+  </si>
+  <si>
+    <t>0.076**</t>
+  </si>
+  <si>
+    <t>0.286</t>
   </si>
   <si>
     <t>0.868***</t>
@@ -415,7 +418,7 @@
         <v>0</v>
       </c>
       <c r="G1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2">
@@ -438,7 +441,7 @@
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3">
@@ -461,7 +464,7 @@
         <v>19</v>
       </c>
       <c r="G3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4">
@@ -481,10 +484,10 @@
         <v>60</v>
       </c>
       <c r="F4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5">
@@ -527,10 +530,10 @@
         <v>62</v>
       </c>
       <c r="F6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7">
@@ -573,10 +576,10 @@
         <v>64</v>
       </c>
       <c r="F8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9">
@@ -619,10 +622,10 @@
         <v>66</v>
       </c>
       <c r="F10" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11">
@@ -665,10 +668,10 @@
         <v>68</v>
       </c>
       <c r="F12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G12" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="13">
@@ -711,10 +714,10 @@
         <v>70</v>
       </c>
       <c r="F14" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="15">
@@ -757,10 +760,10 @@
         <v>72</v>
       </c>
       <c r="F16" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G16" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17">
@@ -803,10 +806,10 @@
         <v>74</v>
       </c>
       <c r="F18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="19">
@@ -849,10 +852,10 @@
         <v>76</v>
       </c>
       <c r="F20" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G20" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21">
@@ -895,10 +898,10 @@
         <v>78</v>
       </c>
       <c r="F22" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G22" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="23">
@@ -941,10 +944,10 @@
         <v>80</v>
       </c>
       <c r="F24" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G24" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="25">
@@ -987,10 +990,10 @@
         <v>82</v>
       </c>
       <c r="F26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G26" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="27">
@@ -1007,7 +1010,7 @@
         <v>0</v>
       </c>
       <c r="E27" t="s">
-        <v>54</v>
+        <v>83</v>
       </c>
       <c r="F27" t="s">
         <v>0</v>
@@ -1030,13 +1033,13 @@
         <v>57</v>
       </c>
       <c r="E28" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F28" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G28" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="29">
@@ -1053,7 +1056,7 @@
         <v>0</v>
       </c>
       <c r="E29" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F29" t="s">
         <v>0</v>
@@ -1076,13 +1079,13 @@
         <v>57</v>
       </c>
       <c r="E30" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F30" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G30" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="31">
@@ -1099,7 +1102,7 @@
         <v>0</v>
       </c>
       <c r="E31" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F31" t="s">
         <v>0</v>
@@ -1122,13 +1125,13 @@
         <v>57</v>
       </c>
       <c r="E32" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F32" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G32" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="33">
@@ -1145,7 +1148,7 @@
         <v>0</v>
       </c>
       <c r="E33" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F33" t="s">
         <v>0</v>
@@ -1168,13 +1171,13 @@
         <v>57</v>
       </c>
       <c r="E34" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F34" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G34" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="35">
@@ -1191,7 +1194,7 @@
         <v>0</v>
       </c>
       <c r="E35" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F35" t="s">
         <v>0</v>

</xml_diff>